<commit_message>
Implementation for ezetap device data decoding
</commit_message>
<xml_diff>
--- a/DataProvider/card_details.xlsx
+++ b/DataProvider/card_details.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="card_details" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -155,7 +155,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.9"/>

</xml_diff>

<commit_message>
Included autologin features and revert autologin in card txns
</commit_message>
<xml_diff>
--- a/DataProvider/card_details.xlsx
+++ b/DataProvider/card_details.xlsx
@@ -5,14 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="card_details" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="bin_info" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">card_details!$A$1:$E$50</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">card_details!$A$1:$E$68</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="103">
   <si>
     <t xml:space="preserve">Transaction Type</t>
   </si>
@@ -56,156 +56,31 @@
     <t xml:space="preserve">ATOS_TLE_EMV_DEBIT_MASTER</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555329</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553298900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMV_DEBIT_RUPAY</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555323</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553238900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMV_CREDIT_VISA</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555324</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553248900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMV_CREDIT_MASTER</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555327</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553278900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMV_CREDIT_RUPAY</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555328</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553288900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_DEBIT_VISA</t>
@@ -217,156 +92,31 @@
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_DEBIT_MASTER</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555329</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553298900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_DEBIT_RUPAY</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555323</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553238900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_CREDIT_VISA</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555324</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553248900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_CREDIT_MASTER</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555327</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553278900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_CREDIT_RUPAY</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE0208</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">555328</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8900833493</t>
-    </r>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553288900833493</t>
   </si>
   <si>
     <t xml:space="preserve">HDFC_EMV_DEBIT_VISA</t>
@@ -477,6 +227,84 @@
     <t xml:space="preserve">FDC_EMVCTLS_CREDIT_RUPAY</t>
   </si>
   <si>
+    <t xml:space="preserve">IDFC_EMV_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMV_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMV_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMV_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMV_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMV_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_EMVCTLS_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_DEBIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553218900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_DEBIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553298900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_DEBIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553238900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_CREDIT_VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553248900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_CREDIT_MASTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDFC_MSR_CREDIT_RUPAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010106FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553288900833493</t>
+  </si>
+  <si>
     <t xml:space="preserve">CONFIRM_DATA</t>
   </si>
   <si>
@@ -498,7 +326,7 @@
     <t xml:space="preserve">DEBIT</t>
   </si>
   <si>
-    <t xml:space="preserve">MASTER</t>
+    <t xml:space="preserve">MASTER_CARD</t>
   </si>
   <si>
     <t xml:space="preserve">RUPAY</t>
@@ -514,7 +342,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -535,11 +363,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -633,8 +456,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
-  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E68"/>
+  <sheetFormatPr defaultColWidth="12.2109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="101.89"/>
@@ -1386,11 +1209,281 @@
         <v>67</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
+      <c r="B51" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1409,20 +1502,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1430,21 +1524,21 @@
         <v>555321</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>555329</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1452,10 +1546,10 @@
         <v>555323</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1463,21 +1557,21 @@
         <v>555324</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
-        <v>555327</v>
+        <v>555325</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1485,10 +1579,10 @@
         <v>555328</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixes wrt to dev16
</commit_message>
<xml_diff>
--- a/DataProvider/card_details.xlsx
+++ b/DataProvider/card_details.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="101">
   <si>
     <t xml:space="preserve">Transaction Type</t>
   </si>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">ATOS_TLE_EMV_CREDIT_MASTER</t>
   </si>
   <si>
-    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553278900833493</t>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMV_CREDIT_RUPAY</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_CREDIT_MASTER</t>
   </si>
   <si>
-    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553278900833493</t>
+    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
   </si>
   <si>
     <t xml:space="preserve">ATOS_TLE_EMVCTLS_CREDIT_RUPAY</t>
@@ -242,9 +242,6 @@
     <t xml:space="preserve">IDFC_EMV_CREDIT_MASTER</t>
   </si>
   <si>
-    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010102FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
-  </si>
-  <si>
     <t xml:space="preserve">IDFC_EMV_CREDIT_RUPAY</t>
   </si>
   <si>
@@ -261,9 +258,6 @@
   </si>
   <si>
     <t xml:space="preserve">IDFC_EMVCTLS_CREDIT_MASTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FE058A820238008407A0000000041010950508400880009A031810119C01005F2A0203565F3401019F02060000000050009F090200029F10120110A00001220000000000000000000000FF9F1A0203569F1E0836413030343234379F260804E65CB7BC82A8A29F2701809F3303E0F0C89F34031E03009F3501229F360201AF9F37049B5EDF7A9F410400000000FE010191FE0803323036FE0910D2F8EA7E5D3D6BD4B29A659DCC111386FE03021808FE0A08CFBB6490E3F1C351FE0D0AFFFF006A004247000404FE061A4E49524F5348412056202020202020202020202020202020202FFE0428B9FE52C1B0E993629389F863C41DFBDA73F3275B2C03AABCAB5853BBB7AD29A0FB20809ACD8D4259FE02085553258900833493</t>
   </si>
   <si>
     <t xml:space="preserve">IDFC_EMVCTLS_CREDIT_RUPAY</t>
@@ -457,10 +451,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E68"/>
-  <sheetFormatPr defaultColWidth="12.2109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="101.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="127.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.06"/>
@@ -814,7 +808,7 @@
       </c>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>41</v>
       </c>
@@ -904,7 +898,7 @@
       </c>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>47</v>
       </c>
@@ -994,7 +988,7 @@
       </c>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>53</v>
       </c>
@@ -1084,7 +1078,7 @@
       </c>
       <c r="E41" s="2"/>
     </row>
-    <row r="42" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>59</v>
       </c>
@@ -1174,7 +1168,7 @@
       </c>
       <c r="E47" s="2"/>
     </row>
-    <row r="48" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>65</v>
       </c>
@@ -1269,7 +1263,7 @@
         <v>71</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
@@ -1281,7 +1275,7 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>18</v>
@@ -1296,7 +1290,7 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>20</v>
@@ -1311,7 +1305,7 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>22</v>
@@ -1326,7 +1320,7 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>24</v>
@@ -1341,7 +1335,7 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>26</v>
@@ -1356,10 +1350,10 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
@@ -1371,7 +1365,7 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>30</v>
@@ -1386,10 +1380,10 @@
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>7</v>
@@ -1401,10 +1395,10 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>7</v>
@@ -1416,10 +1410,10 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>7</v>
@@ -1431,10 +1425,10 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>7</v>
@@ -1446,10 +1440,10 @@
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>7</v>
@@ -1461,10 +1455,10 @@
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>7</v>
@@ -1476,10 +1470,10 @@
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
@@ -1502,7 +1496,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.52"/>
@@ -1510,13 +1504,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1524,10 +1518,10 @@
         <v>555321</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1535,10 +1529,10 @@
         <v>555329</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1546,10 +1540,10 @@
         <v>555323</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1557,10 +1551,10 @@
         <v>555324</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1568,10 +1562,10 @@
         <v>555325</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1579,10 +1573,10 @@
         <v>555328</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TID dep AXIS_ATOS BQRV4 UPI
</commit_message>
<xml_diff>
--- a/DataProvider/card_details.xlsx
+++ b/DataProvider/card_details.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="card_details" sheetId="1" state="visible" r:id="rId2"/>
@@ -451,7 +451,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E68"/>
-  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="127.46"/>
@@ -1496,7 +1496,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.52"/>

</xml_diff>